<commit_message>
research(pass2c): run targeted lane probes and update conformance status
</commit_message>
<xml_diff>
--- a/research/runs/20260302-070309-excel-formula-language-pass2-pack-01/fixtures/formula_parse_pass2/Book2.xlsx
+++ b/research/runs/20260302-070309-excel-formula-language-pass2-pack-01/fixtures/formula_parse_pass2/Book2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\DnaCalc\Foundation\research\runs\20260302-070309-excel-formula-language-pass2-pack-01\fixtures\formula_parse_pass2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{221CDFF0-E2E4-4805-8BDF-8D0D2770707A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{896E0180-7F8D-4D7C-866B-6DED672B3076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3135" yWindow="3885" windowWidth="11955" windowHeight="11595" xr2:uid="{83AEAA57-420B-4C2F-BF88-33340C384E87}"/>
+    <workbookView xWindow="3135" yWindow="3885" windowWidth="11955" windowHeight="11595" xr2:uid="{D1B2E49C-A9EB-490D-9446-50E4B69A968C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -401,7 +401,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6428834F-B074-42CC-B4F1-557DA391C70C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40745F62-6AF6-4C3E-ACA1-329A1D58863E}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>